<commit_message>
UPDATE: New WS, RS, Alvez Pricelist, and added angpao for voucher giias column
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8626274-3E33-48DC-967C-B4755BBB7B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3CFD31-6A96-46C9-A31C-BE51EF926D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -490,7 +490,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1375" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="618">
   <si>
     <t>Column1</t>
   </si>
@@ -2408,10 +2408,22 @@
     <t>NEW ALVEZ CE MT 310S I1F1 (4X2) M/T</t>
   </si>
   <si>
-    <t>New Alvez 1.5 CE 4X2 CVT</t>
-  </si>
-  <si>
     <t>Cortez (NEW CORTEZ CE LUX+CVT) LT +CVT</t>
+  </si>
+  <si>
+    <t>NEW ALVEZ CE AT 310S I2F1 (4X2) A/T</t>
+  </si>
+  <si>
+    <t>New Alvez CE MT</t>
+  </si>
+  <si>
+    <t>New Alvez CE AT</t>
+  </si>
+  <si>
+    <t>NEW ALVEZ CE AT 310S I2D1 (4X2) A/T</t>
+  </si>
+  <si>
+    <t>New Alvez EX AT</t>
   </si>
 </sst>
 </file>
@@ -2603,7 +2615,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2638,9 +2650,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2648,6 +2657,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -5022,10 +5033,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I54" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
-  <autoFilter ref="A1:I54" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I54">
-    <sortCondition ref="H1:H54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I56" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
+  <autoFilter ref="A1:I56" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I56">
+    <sortCondition ref="H1:H56"/>
   </sortState>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="149"/>
@@ -5651,7 +5662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B05C9E0-A64E-40AC-B9F4-C919ED5906CC}">
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
@@ -5726,15 +5737,15 @@
         <v>214000000</v>
       </c>
       <c r="D2" s="5">
-        <f>I2/1.12</f>
+        <f t="shared" ref="D2:D35" si="0">I2/1.12</f>
         <v>18750000</v>
       </c>
       <c r="E2" s="5">
-        <f>D2*90%</f>
+        <f t="shared" ref="E2:E35" si="1">D2*90%</f>
         <v>16875000</v>
       </c>
       <c r="F2" s="5">
-        <f>D2*70%</f>
+        <f t="shared" ref="F2:F35" si="2">D2*70%</f>
         <v>13125000</v>
       </c>
       <c r="G2" s="3">
@@ -5758,15 +5769,15 @@
         <v>251000000</v>
       </c>
       <c r="D3" s="5">
-        <f>I3/1.12</f>
+        <f t="shared" si="0"/>
         <v>18750000</v>
       </c>
       <c r="E3" s="5">
-        <f>D3*90%</f>
+        <f t="shared" si="1"/>
         <v>16875000</v>
       </c>
       <c r="F3" s="5">
-        <f>D3*70%</f>
+        <f t="shared" si="2"/>
         <v>13125000</v>
       </c>
       <c r="G3" s="3">
@@ -5790,15 +5801,15 @@
         <v>251000000</v>
       </c>
       <c r="D4" s="5">
-        <f>I4/1.12</f>
+        <f t="shared" si="0"/>
         <v>18750000</v>
       </c>
       <c r="E4" s="5">
-        <f>D4*90%</f>
+        <f t="shared" si="1"/>
         <v>16875000</v>
       </c>
       <c r="F4" s="5">
-        <f>D4*70%</f>
+        <f t="shared" si="2"/>
         <v>13125000</v>
       </c>
       <c r="G4" s="3">
@@ -5822,15 +5833,15 @@
         <v>251000000</v>
       </c>
       <c r="D5" s="5">
-        <f>I5/1.12</f>
+        <f t="shared" si="0"/>
         <v>18750000</v>
       </c>
       <c r="E5" s="5">
-        <f>D5*90%</f>
+        <f t="shared" si="1"/>
         <v>16875000</v>
       </c>
       <c r="F5" s="5">
-        <f>D5*70%</f>
+        <f t="shared" si="2"/>
         <v>13125000</v>
       </c>
       <c r="G5" s="3">
@@ -5854,15 +5865,15 @@
         <v>307500000</v>
       </c>
       <c r="D6" s="5">
-        <f>I6/1.12</f>
+        <f t="shared" si="0"/>
         <v>22321428.571428567</v>
       </c>
       <c r="E6" s="5">
-        <f>D6*90%</f>
+        <f t="shared" si="1"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F6" s="5">
-        <f>D6*70%</f>
+        <f t="shared" si="2"/>
         <v>15624999.999999996</v>
       </c>
       <c r="G6" s="3">
@@ -5886,15 +5897,15 @@
         <v>311500000</v>
       </c>
       <c r="D7" s="5">
-        <f>I7/1.12</f>
+        <f t="shared" si="0"/>
         <v>20758928.571428567</v>
       </c>
       <c r="E7" s="5">
-        <f>D7*90%</f>
+        <f t="shared" si="1"/>
         <v>18683035.714285713</v>
       </c>
       <c r="F7" s="5">
-        <f>D7*70%</f>
+        <f t="shared" si="2"/>
         <v>14531249.999999996</v>
       </c>
       <c r="G7" s="7">
@@ -5918,15 +5929,15 @@
         <v>329050000</v>
       </c>
       <c r="D8" s="5">
-        <f>I8/1.12</f>
+        <f t="shared" si="0"/>
         <v>22053571.428571429</v>
       </c>
       <c r="E8" s="5">
-        <f>D8*90%</f>
+        <f t="shared" si="1"/>
         <v>19848214.285714287</v>
       </c>
       <c r="F8" s="5">
-        <f>D8*70%</f>
+        <f t="shared" si="2"/>
         <v>15437500</v>
       </c>
       <c r="G8" s="7">
@@ -5950,15 +5961,15 @@
         <v>388500000</v>
       </c>
       <c r="D9" s="5">
-        <f>I9/1.12</f>
+        <f t="shared" si="0"/>
         <v>29464285.714285709</v>
       </c>
       <c r="E9" s="5">
-        <f>D9*90%</f>
+        <f t="shared" si="1"/>
         <v>26517857.142857138</v>
       </c>
       <c r="F9" s="5">
-        <f>D9*70%</f>
+        <f t="shared" si="2"/>
         <v>20624999.999999996</v>
       </c>
       <c r="G9" s="7">
@@ -5982,15 +5993,15 @@
         <v>447200000</v>
       </c>
       <c r="D10" s="5">
-        <f>I10/1.12</f>
+        <f t="shared" si="0"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E10" s="5">
-        <f>D10*90%</f>
+        <f t="shared" si="1"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F10" s="5">
-        <f>D10*70%</f>
+        <f t="shared" si="2"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G10" s="7">
@@ -6014,15 +6025,15 @@
         <v>405000000</v>
       </c>
       <c r="D11" s="5">
-        <f>I11/1.12</f>
+        <f t="shared" si="0"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E11" s="5">
-        <f>D11*90%</f>
+        <f t="shared" si="1"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F11" s="5">
-        <f>D11*70%</f>
+        <f t="shared" si="2"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G11" s="7">
@@ -6046,15 +6057,15 @@
         <v>442000000</v>
       </c>
       <c r="D12" s="5">
-        <f>I12/1.12</f>
+        <f t="shared" si="0"/>
         <v>33928571.428571425</v>
       </c>
       <c r="E12" s="5">
-        <f>D12*90%</f>
+        <f t="shared" si="1"/>
         <v>30535714.285714284</v>
       </c>
       <c r="F12" s="5">
-        <f>D12*70%</f>
+        <f t="shared" si="2"/>
         <v>23749999.999999996</v>
       </c>
       <c r="G12" s="7">
@@ -6078,15 +6089,15 @@
         <v>303000000</v>
       </c>
       <c r="D13" s="5">
-        <f>I13/1.12</f>
+        <f t="shared" si="0"/>
         <v>20535714.285714284</v>
       </c>
       <c r="E13" s="5">
-        <f>D13*90%</f>
+        <f t="shared" si="1"/>
         <v>18482142.857142854</v>
       </c>
       <c r="F13" s="5">
-        <f>D13*70%</f>
+        <f t="shared" si="2"/>
         <v>14374999.999999998</v>
       </c>
       <c r="G13" s="3">
@@ -6110,15 +6121,15 @@
         <v>263000000</v>
       </c>
       <c r="D14" s="5">
-        <f>I14/1.12</f>
+        <f t="shared" si="0"/>
         <v>17857142.857142854</v>
       </c>
       <c r="E14" s="5">
-        <f>D14*90%</f>
+        <f t="shared" si="1"/>
         <v>16071428.571428569</v>
       </c>
       <c r="F14" s="5">
-        <f>D14*70%</f>
+        <f t="shared" si="2"/>
         <v>12499999.999999998</v>
       </c>
       <c r="G14" s="3">
@@ -6142,15 +6153,15 @@
         <v>217000000</v>
       </c>
       <c r="D15" s="5">
-        <f>I15/1.12</f>
+        <f t="shared" si="0"/>
         <v>11607142.857142856</v>
       </c>
       <c r="E15" s="5">
-        <f>D15*90%</f>
+        <f t="shared" si="1"/>
         <v>10446428.571428571</v>
       </c>
       <c r="F15" s="5">
-        <f>D15*70%</f>
+        <f t="shared" si="2"/>
         <v>8124999.9999999991</v>
       </c>
       <c r="G15" s="3">
@@ -6164,26 +6175,26 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="10" t="s">
         <v>611</v>
       </c>
-      <c r="B16" s="23" t="s">
-        <v>612</v>
+      <c r="B16" s="4" t="s">
+        <v>614</v>
       </c>
       <c r="C16" s="5">
-        <v>263000000</v>
+        <v>217000000</v>
       </c>
       <c r="D16" s="5">
-        <f>I16/1.12</f>
-        <v>17857142.857142854</v>
+        <f t="shared" si="0"/>
+        <v>11607142.857142856</v>
       </c>
       <c r="E16" s="5">
-        <f>D16*90%</f>
-        <v>16071428.571428569</v>
+        <f t="shared" si="1"/>
+        <v>10446428.571428571</v>
       </c>
       <c r="F16" s="5">
-        <f>D16*70%</f>
-        <v>12499999.999999998</v>
+        <f t="shared" si="2"/>
+        <v>8124999.9999999991</v>
       </c>
       <c r="G16" s="3">
         <v>262</v>
@@ -6192,268 +6203,268 @@
         <v>566</v>
       </c>
       <c r="I16" s="12">
+        <v>13000000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="25" t="s">
+        <v>613</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>615</v>
+      </c>
+      <c r="C17" s="5">
+        <v>263000000</v>
+      </c>
+      <c r="D17" s="5">
+        <f t="shared" ref="D17" si="3">I17/1.12</f>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E17" s="5">
+        <f t="shared" si="1"/>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F17" s="5">
+        <f t="shared" ref="F17" si="4">D17*70%</f>
+        <v>12499999.999999998</v>
+      </c>
+      <c r="G17" s="3">
+        <v>263</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="I17" s="12">
         <v>20000000</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
-        <v>503</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>549</v>
-      </c>
-      <c r="C17" s="5">
-        <v>353000000</v>
-      </c>
-      <c r="D17" s="5">
-        <f>I17/1.12</f>
-        <v>25892857.142857142</v>
-      </c>
-      <c r="E17" s="5">
-        <f>D17*90%</f>
-        <v>23303571.428571429</v>
-      </c>
-      <c r="F17" s="5">
-        <f>D17*70%</f>
-        <v>18124999.999999996</v>
-      </c>
-      <c r="G17" s="3">
-        <v>246</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="I17" s="12">
-        <v>29000000</v>
-      </c>
-    </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
-        <v>586</v>
+      <c r="A18" s="25" t="s">
+        <v>616</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>583</v>
-      </c>
-      <c r="C18" s="5">
-        <v>318000000</v>
+        <v>617</v>
+      </c>
+      <c r="C18" s="9">
+        <v>303000000</v>
       </c>
       <c r="D18" s="5">
-        <f>I18/1.12</f>
-        <v>23214285.714285713</v>
+        <f t="shared" ref="D18" si="5">I18/1.12</f>
+        <v>20535714.285714284</v>
       </c>
       <c r="E18" s="5">
-        <f>D18*90%</f>
-        <v>20892857.142857142</v>
+        <f t="shared" si="1"/>
+        <v>18482142.857142854</v>
       </c>
       <c r="F18" s="5">
-        <f>D18*70%</f>
-        <v>16249999.999999998</v>
+        <f t="shared" ref="F18" si="6">D18*70%</f>
+        <v>14374999.999999998</v>
       </c>
       <c r="G18" s="3">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="I18" s="12">
-        <v>26000000</v>
+        <v>566</v>
+      </c>
+      <c r="I18" s="26">
+        <v>23000000</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>510</v>
+        <v>549</v>
       </c>
       <c r="C19" s="5">
-        <v>363000000</v>
+        <v>353000000</v>
       </c>
       <c r="D19" s="5">
-        <f>I19/1.12</f>
-        <v>26785714.285714284</v>
+        <f t="shared" si="0"/>
+        <v>25892857.142857142</v>
       </c>
       <c r="E19" s="5">
-        <f>D19*90%</f>
-        <v>24107142.857142854</v>
+        <f t="shared" si="1"/>
+        <v>23303571.428571429</v>
       </c>
       <c r="F19" s="5">
-        <f>D19*70%</f>
-        <v>18749999.999999996</v>
+        <f t="shared" si="2"/>
+        <v>18124999.999999996</v>
       </c>
       <c r="G19" s="3">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="I19" s="12">
-        <v>30000000</v>
+        <v>29000000</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="C20" s="5">
-        <v>363000000</v>
+        <v>318000000</v>
       </c>
       <c r="D20" s="5">
-        <f>I20/1.12</f>
-        <v>25892857.142857142</v>
+        <f t="shared" si="0"/>
+        <v>23214285.714285713</v>
       </c>
       <c r="E20" s="5">
-        <f>D20*90%</f>
-        <v>23303571.428571429</v>
+        <f t="shared" si="1"/>
+        <v>20892857.142857142</v>
       </c>
       <c r="F20" s="5">
-        <f>D20*70%</f>
-        <v>18124999.999999996</v>
+        <f t="shared" si="2"/>
+        <v>16249999.999999998</v>
       </c>
       <c r="G20" s="3">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="I20" s="12">
-        <v>29000000</v>
+        <v>26000000</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
-        <v>587</v>
+        <v>504</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>584</v>
+        <v>510</v>
       </c>
       <c r="C21" s="5">
         <v>363000000</v>
       </c>
       <c r="D21" s="5">
-        <f>I21/1.12</f>
-        <v>25892857.142857142</v>
+        <f t="shared" si="0"/>
+        <v>26785714.285714284</v>
       </c>
       <c r="E21" s="5">
-        <f>D21*90%</f>
-        <v>23303571.428571429</v>
+        <f t="shared" si="1"/>
+        <v>24107142.857142854</v>
       </c>
       <c r="F21" s="5">
-        <f>D21*70%</f>
-        <v>18124999.999999996</v>
+        <f t="shared" si="2"/>
+        <v>18749999.999999996</v>
       </c>
       <c r="G21" s="3">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>577</v>
       </c>
       <c r="I21" s="12">
-        <v>29000000</v>
+        <v>30000000</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
-        <v>505</v>
+        <v>588</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>511</v>
+        <v>584</v>
       </c>
       <c r="C22" s="5">
-        <v>413000000</v>
+        <v>363000000</v>
       </c>
       <c r="D22" s="5">
-        <f>I22/1.12</f>
-        <v>30357142.857142854</v>
+        <f t="shared" si="0"/>
+        <v>25892857.142857142</v>
       </c>
       <c r="E22" s="5">
-        <f>D22*90%</f>
-        <v>27321428.571428571</v>
+        <f t="shared" si="1"/>
+        <v>23303571.428571429</v>
       </c>
       <c r="F22" s="5">
-        <f>D22*70%</f>
-        <v>21249999.999999996</v>
+        <f t="shared" si="2"/>
+        <v>18124999.999999996</v>
       </c>
       <c r="G22" s="3">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="I22" s="12">
-        <v>34000000</v>
+        <v>29000000</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
-        <v>558</v>
+        <v>587</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>512</v>
+        <v>584</v>
       </c>
       <c r="C23" s="5">
-        <v>443000000</v>
+        <v>363000000</v>
       </c>
       <c r="D23" s="5">
-        <f>I23/1.12</f>
-        <v>33035714.285714284</v>
+        <f t="shared" si="0"/>
+        <v>25892857.142857142</v>
       </c>
       <c r="E23" s="5">
-        <f>D23*90%</f>
-        <v>29732142.857142854</v>
+        <f t="shared" si="1"/>
+        <v>23303571.428571429</v>
       </c>
       <c r="F23" s="5">
-        <f>D23*70%</f>
-        <v>23124999.999999996</v>
+        <f t="shared" si="2"/>
+        <v>18124999.999999996</v>
       </c>
       <c r="G23" s="3">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="I23" s="12">
-        <v>37000000</v>
+        <v>29000000</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C24" s="5">
-        <v>443000000</v>
+        <v>413000000</v>
       </c>
       <c r="D24" s="5">
-        <f>I24/1.12</f>
-        <v>33035714.285714284</v>
+        <f t="shared" si="0"/>
+        <v>30357142.857142854</v>
       </c>
       <c r="E24" s="5">
-        <f>D24*90%</f>
-        <v>29732142.857142854</v>
+        <f t="shared" si="1"/>
+        <v>27321428.571428571</v>
       </c>
       <c r="F24" s="5">
-        <f>D24*70%</f>
-        <v>23124999.999999996</v>
+        <f t="shared" si="2"/>
+        <v>21249999.999999996</v>
       </c>
       <c r="G24" s="3">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="I24" s="12">
-        <v>37000000</v>
+        <v>34000000</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>512</v>
@@ -6462,15 +6473,15 @@
         <v>443000000</v>
       </c>
       <c r="D25" s="5">
-        <f>I25/1.12</f>
+        <f t="shared" si="0"/>
         <v>33035714.285714284</v>
       </c>
       <c r="E25" s="5">
-        <f>D25*90%</f>
+        <f t="shared" si="1"/>
         <v>29732142.857142854</v>
       </c>
       <c r="F25" s="5">
-        <f>D25*70%</f>
+        <f t="shared" si="2"/>
         <v>23124999.999999996</v>
       </c>
       <c r="G25" s="3">
@@ -6485,31 +6496,31 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
-        <v>557</v>
+        <v>506</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>559</v>
+        <v>512</v>
       </c>
       <c r="C26" s="5">
-        <v>415000000</v>
+        <v>443000000</v>
       </c>
       <c r="D26" s="5">
-        <f>I26/1.12</f>
+        <f t="shared" si="0"/>
         <v>33035714.285714284</v>
       </c>
       <c r="E26" s="5">
-        <f>D26*90%</f>
+        <f t="shared" si="1"/>
         <v>29732142.857142854</v>
       </c>
       <c r="F26" s="5">
-        <f>D26*70%</f>
+        <f t="shared" si="2"/>
         <v>23124999.999999996</v>
       </c>
       <c r="G26" s="3">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>581</v>
+        <v>571</v>
       </c>
       <c r="I26" s="12">
         <v>37000000</v>
@@ -6517,31 +6528,31 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
-        <v>582</v>
+        <v>561</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>559</v>
+        <v>512</v>
       </c>
       <c r="C27" s="5">
-        <v>415000000</v>
+        <v>443000000</v>
       </c>
       <c r="D27" s="5">
-        <f>I27/1.12</f>
+        <f t="shared" si="0"/>
         <v>33035714.285714284</v>
       </c>
       <c r="E27" s="5">
-        <f>D27*90%</f>
+        <f t="shared" si="1"/>
         <v>29732142.857142854</v>
       </c>
       <c r="F27" s="5">
-        <f>D27*70%</f>
+        <f t="shared" si="2"/>
         <v>23124999.999999996</v>
       </c>
       <c r="G27" s="3">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>581</v>
+        <v>571</v>
       </c>
       <c r="I27" s="12">
         <v>37000000</v>
@@ -6549,447 +6560,447 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
-        <v>523</v>
+        <v>557</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>535</v>
+        <v>559</v>
       </c>
       <c r="C28" s="5">
-        <v>188300000</v>
+        <v>415000000</v>
       </c>
       <c r="D28" s="5">
-        <f>I28/1.12</f>
-        <v>11339285.714285715</v>
+        <f t="shared" si="0"/>
+        <v>33035714.285714284</v>
       </c>
       <c r="E28" s="5">
-        <f>D28*90%</f>
-        <v>10205357.142857144</v>
+        <f t="shared" si="1"/>
+        <v>29732142.857142854</v>
       </c>
       <c r="F28" s="5">
-        <f>D28*70%</f>
-        <v>7937500</v>
+        <f t="shared" si="2"/>
+        <v>23124999.999999996</v>
       </c>
       <c r="G28" s="3">
-        <v>202</v>
+        <v>251</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>568</v>
+        <v>581</v>
       </c>
       <c r="I28" s="12">
-        <v>12700000.000000002</v>
+        <v>37000000</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
-        <v>560</v>
+        <v>582</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>535</v>
+        <v>559</v>
       </c>
       <c r="C29" s="5">
-        <v>188300000</v>
+        <v>415000000</v>
       </c>
       <c r="D29" s="5">
-        <f>I29/1.12</f>
-        <v>11339285.714285715</v>
+        <f t="shared" si="0"/>
+        <v>33035714.285714284</v>
       </c>
       <c r="E29" s="5">
-        <f>D29*90%</f>
-        <v>10205357.142857144</v>
+        <f t="shared" si="1"/>
+        <v>29732142.857142854</v>
       </c>
       <c r="F29" s="5">
-        <f>D29*70%</f>
-        <v>7937500</v>
+        <f t="shared" si="2"/>
+        <v>23124999.999999996</v>
       </c>
       <c r="G29" s="3">
-        <v>202</v>
+        <v>251</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>568</v>
+        <v>581</v>
       </c>
       <c r="I29" s="12">
-        <v>12700000.000000002</v>
+        <v>37000000</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C30" s="5">
-        <v>222850000</v>
+        <v>188300000</v>
       </c>
       <c r="D30" s="5">
-        <f>I30/1.12</f>
-        <v>14285714.285714284</v>
+        <f t="shared" si="0"/>
+        <v>11339285.714285715</v>
       </c>
       <c r="E30" s="5">
-        <f>D30*90%</f>
-        <v>12857142.857142856</v>
+        <f t="shared" si="1"/>
+        <v>10205357.142857144</v>
       </c>
       <c r="F30" s="5">
-        <f>D30*70%</f>
-        <v>9999999.9999999981</v>
+        <f t="shared" si="2"/>
+        <v>7937500</v>
       </c>
       <c r="G30" s="3">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>573</v>
+        <v>568</v>
       </c>
       <c r="I30" s="12">
-        <v>16000000</v>
+        <v>12700000.000000002</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
-        <v>498</v>
+        <v>560</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C31" s="5">
-        <v>210700000</v>
+        <v>188300000</v>
       </c>
       <c r="D31" s="5">
-        <f>I31/1.12</f>
-        <v>13124999.999999998</v>
+        <f t="shared" si="0"/>
+        <v>11339285.714285715</v>
       </c>
       <c r="E31" s="5">
-        <f>D31*90%</f>
-        <v>11812499.999999998</v>
+        <f t="shared" si="1"/>
+        <v>10205357.142857144</v>
       </c>
       <c r="F31" s="5">
-        <f>D31*70%</f>
-        <v>9187499.9999999981</v>
+        <f t="shared" si="2"/>
+        <v>7937500</v>
       </c>
       <c r="G31" s="3">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>573</v>
+        <v>568</v>
       </c>
       <c r="I31" s="12">
-        <v>14700000</v>
+        <v>12700000.000000002</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="10" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="C32" s="5">
-        <v>262500000</v>
+        <v>222850000</v>
       </c>
       <c r="D32" s="5">
-        <f>I32/1.12</f>
-        <v>16339285.714285713</v>
+        <f t="shared" si="0"/>
+        <v>14285714.285714284</v>
       </c>
       <c r="E32" s="5">
-        <f>D32*90%</f>
-        <v>14705357.142857142</v>
+        <f t="shared" si="1"/>
+        <v>12857142.857142856</v>
       </c>
       <c r="F32" s="5">
-        <f>D32*70%</f>
-        <v>11437499.999999998</v>
+        <f t="shared" si="2"/>
+        <v>9999999.9999999981</v>
       </c>
       <c r="G32" s="3">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="I32" s="12">
-        <v>18300000</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
-        <v>527</v>
+        <v>498</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>490</v>
+        <v>537</v>
       </c>
       <c r="C33" s="5">
-        <v>277200000</v>
+        <v>210700000</v>
       </c>
       <c r="D33" s="5">
-        <f>I33/1.12</f>
-        <v>18660714.285714284</v>
+        <f t="shared" si="0"/>
+        <v>13124999.999999998</v>
       </c>
       <c r="E33" s="5">
-        <f>D33*90%</f>
-        <v>16794642.857142854</v>
+        <f t="shared" si="1"/>
+        <v>11812499.999999998</v>
       </c>
       <c r="F33" s="5">
-        <f>D33*70%</f>
-        <v>13062499.999999998</v>
+        <f t="shared" si="2"/>
+        <v>9187499.9999999981</v>
       </c>
       <c r="G33" s="3">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="I33" s="12">
-        <v>20900000</v>
+        <v>14700000</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>491</v>
+        <v>544</v>
       </c>
       <c r="C34" s="5">
-        <v>291300000</v>
+        <v>262500000</v>
       </c>
       <c r="D34" s="5">
-        <f>I34/1.12</f>
-        <v>19642857.142857142</v>
+        <f t="shared" si="0"/>
+        <v>16339285.714285713</v>
       </c>
       <c r="E34" s="5">
-        <f>D34*90%</f>
-        <v>17678571.428571429</v>
+        <f t="shared" si="1"/>
+        <v>14705357.142857142</v>
       </c>
       <c r="F34" s="5">
-        <f>D34*70%</f>
-        <v>13749999.999999998</v>
+        <f t="shared" si="2"/>
+        <v>11437499.999999998</v>
       </c>
       <c r="G34" s="3">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="H34" s="4" t="s">
         <v>567</v>
       </c>
       <c r="I34" s="12">
-        <v>22000000</v>
+        <v>18300000</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
-        <v>499</v>
+        <v>527</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="C35" s="5">
-        <v>285200000</v>
+        <v>277200000</v>
       </c>
       <c r="D35" s="5">
-        <f>I35/1.12</f>
-        <v>18303571.428571429</v>
+        <f t="shared" si="0"/>
+        <v>18660714.285714284</v>
       </c>
       <c r="E35" s="5">
-        <f>D35*90%</f>
-        <v>16473214.285714287</v>
+        <f t="shared" si="1"/>
+        <v>16794642.857142854</v>
       </c>
       <c r="F35" s="5">
-        <f>D35*70%</f>
-        <v>12812500</v>
+        <f t="shared" si="2"/>
+        <v>13062499.999999998</v>
       </c>
       <c r="G35" s="3">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="H35" s="4" t="s">
         <v>567</v>
       </c>
       <c r="I35" s="12">
-        <v>20500000.000000004</v>
+        <v>20900000</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A36" s="11" t="s">
-        <v>522</v>
+      <c r="A36" s="10" t="s">
+        <v>528</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>550</v>
+        <v>491</v>
       </c>
       <c r="C36" s="5">
-        <v>345650000</v>
+        <v>291300000</v>
       </c>
       <c r="D36" s="5">
-        <f>I36/1.12</f>
-        <v>22857142.857142854</v>
+        <f t="shared" ref="D36:D56" si="7">I36/1.12</f>
+        <v>19642857.142857142</v>
       </c>
       <c r="E36" s="5">
-        <f>D36*90%</f>
-        <v>20571428.571428571</v>
+        <f t="shared" ref="E36:E67" si="8">D36*90%</f>
+        <v>17678571.428571429</v>
       </c>
       <c r="F36" s="5">
-        <f>D36*70%</f>
-        <v>15999999.999999996</v>
+        <f t="shared" ref="F36:F56" si="9">D36*70%</f>
+        <v>13749999.999999998</v>
       </c>
       <c r="G36" s="3">
-        <v>233</v>
+        <v>214</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>567</v>
       </c>
       <c r="I36" s="12">
-        <v>25600000</v>
+        <v>22000000</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A37" s="25" t="s">
-        <v>149</v>
-      </c>
-      <c r="B37" s="23" t="s">
-        <v>613</v>
-      </c>
-      <c r="C37" s="9">
-        <v>307300000</v>
+      <c r="A37" s="10" t="s">
+        <v>499</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="C37" s="5">
+        <v>285200000</v>
       </c>
       <c r="D37" s="5">
-        <f>I37/1.12</f>
-        <v>19999999.999999996</v>
+        <f t="shared" si="7"/>
+        <v>18303571.428571429</v>
       </c>
       <c r="E37" s="5">
-        <f>D37*90%</f>
-        <v>17999999.999999996</v>
+        <f t="shared" si="8"/>
+        <v>16473214.285714287</v>
       </c>
       <c r="F37" s="5">
-        <f>D37*70%</f>
-        <v>13999999.999999996</v>
-      </c>
-      <c r="G37" s="4">
-        <v>210</v>
+        <f t="shared" si="9"/>
+        <v>12812500</v>
+      </c>
+      <c r="G37" s="3">
+        <v>220</v>
       </c>
       <c r="H37" s="4" t="s">
         <v>567</v>
       </c>
-      <c r="I37" s="24">
+      <c r="I37" s="12">
+        <v>20500000.000000004</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38" s="11" t="s">
+        <v>522</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="C38" s="5">
+        <v>345650000</v>
+      </c>
+      <c r="D38" s="5">
+        <f t="shared" si="7"/>
+        <v>22857142.857142854</v>
+      </c>
+      <c r="E38" s="5">
+        <f t="shared" si="8"/>
+        <v>20571428.571428571</v>
+      </c>
+      <c r="F38" s="5">
+        <f t="shared" si="9"/>
+        <v>15999999.999999996</v>
+      </c>
+      <c r="G38" s="3">
+        <v>233</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="I38" s="12">
+        <v>25600000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>612</v>
+      </c>
+      <c r="C39" s="9">
+        <v>307300000</v>
+      </c>
+      <c r="D39" s="5">
+        <f t="shared" si="7"/>
+        <v>19999999.999999996</v>
+      </c>
+      <c r="E39" s="5">
+        <f t="shared" si="8"/>
+        <v>17999999.999999996</v>
+      </c>
+      <c r="F39" s="5">
+        <f t="shared" si="9"/>
+        <v>13999999.999999996</v>
+      </c>
+      <c r="G39" s="4">
+        <v>210</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="I39" s="12">
         <v>22400000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A38" s="10" t="s">
-        <v>608</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>597</v>
-      </c>
-      <c r="C38" s="9">
-        <v>399000000</v>
-      </c>
-      <c r="D38" s="9">
-        <f>I38/1.12</f>
-        <v>28214285.714285713</v>
-      </c>
-      <c r="E38" s="9">
-        <f>D38*90%</f>
-        <v>25392857.142857142</v>
-      </c>
-      <c r="F38" s="9">
-        <f>D38*70%</f>
-        <v>19749999.999999996</v>
-      </c>
-      <c r="G38" s="20">
-        <v>258</v>
-      </c>
-      <c r="H38" s="4" t="s">
-        <v>597</v>
-      </c>
-      <c r="I38" s="12">
-        <v>31600000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
-        <v>599</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>598</v>
-      </c>
-      <c r="C39" s="9">
-        <v>459000000</v>
-      </c>
-      <c r="D39" s="9">
-        <f>I39/1.12</f>
-        <v>32499999.999999996</v>
-      </c>
-      <c r="E39" s="9">
-        <f>D39*90%</f>
-        <v>29249999.999999996</v>
-      </c>
-      <c r="F39" s="9">
-        <f>D39*70%</f>
-        <v>22749999.999999996</v>
-      </c>
-      <c r="G39" s="20">
-        <v>259</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>598</v>
-      </c>
-      <c r="I39" s="12">
-        <v>36400000</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" s="10" t="s">
-        <v>601</v>
+        <v>608</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="C40" s="9">
-        <v>449000000</v>
+        <v>399000000</v>
       </c>
       <c r="D40" s="9">
-        <f>I40/1.12</f>
-        <v>29196428.571428567</v>
+        <f t="shared" si="7"/>
+        <v>28214285.714285713</v>
       </c>
       <c r="E40" s="9">
-        <f>D40*90%</f>
-        <v>26276785.714285713</v>
+        <f t="shared" si="8"/>
+        <v>25392857.142857142</v>
       </c>
       <c r="F40" s="9">
-        <f>D40*70%</f>
-        <v>20437499.999999996</v>
+        <f t="shared" si="9"/>
+        <v>19749999.999999996</v>
       </c>
       <c r="G40" s="20">
-        <v>260</v>
-      </c>
-      <c r="H40" s="10" t="s">
-        <v>600</v>
+        <v>258</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>597</v>
       </c>
       <c r="I40" s="12">
-        <v>32700000</v>
+        <v>31600000</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="C41" s="9">
-        <v>499000000</v>
+        <v>459000000</v>
       </c>
       <c r="D41" s="9">
-        <f>I41/1.12</f>
+        <f t="shared" si="7"/>
         <v>32499999.999999996</v>
       </c>
       <c r="E41" s="9">
-        <f>D41*90%</f>
+        <f t="shared" si="8"/>
         <v>29249999.999999996</v>
       </c>
       <c r="F41" s="9">
-        <f>D41*70%</f>
+        <f t="shared" si="9"/>
         <v>22749999.999999996</v>
       </c>
       <c r="G41" s="20">
-        <v>261</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>602</v>
+        <v>259</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>598</v>
       </c>
       <c r="I41" s="12">
         <v>36400000</v>
@@ -6997,417 +7008,481 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
+        <v>601</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="C42" s="9">
+        <v>449000000</v>
+      </c>
+      <c r="D42" s="9">
+        <f t="shared" si="7"/>
+        <v>29196428.571428567</v>
+      </c>
+      <c r="E42" s="9">
+        <f t="shared" si="8"/>
+        <v>26276785.714285713</v>
+      </c>
+      <c r="F42" s="9">
+        <f t="shared" si="9"/>
+        <v>20437499.999999996</v>
+      </c>
+      <c r="G42" s="20">
+        <v>260</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>600</v>
+      </c>
+      <c r="I42" s="12">
+        <v>32700000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43" s="10" t="s">
+        <v>603</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>602</v>
+      </c>
+      <c r="C43" s="9">
+        <v>499000000</v>
+      </c>
+      <c r="D43" s="9">
+        <f t="shared" si="7"/>
+        <v>32499999.999999996</v>
+      </c>
+      <c r="E43" s="9">
+        <f t="shared" si="8"/>
+        <v>29249999.999999996</v>
+      </c>
+      <c r="F43" s="9">
+        <f t="shared" si="9"/>
+        <v>22749999.999999996</v>
+      </c>
+      <c r="G43" s="20">
+        <v>261</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>602</v>
+      </c>
+      <c r="I43" s="12">
+        <v>36400000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44" s="10" t="s">
         <v>526</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B44" s="4" t="s">
         <v>545</v>
       </c>
-      <c r="C42" s="5">
+      <c r="C44" s="5">
         <v>168000000</v>
       </c>
-      <c r="D42" s="5">
-        <f>I42/1.12</f>
+      <c r="D44" s="5">
+        <f t="shared" si="7"/>
         <v>11160714.285714284</v>
       </c>
-      <c r="E42" s="5">
-        <f>D42*90%</f>
+      <c r="E44" s="5">
+        <f t="shared" si="8"/>
         <v>10044642.857142856</v>
       </c>
-      <c r="F42" s="5">
-        <f>D42*70%</f>
+      <c r="F44" s="5">
+        <f t="shared" si="9"/>
         <v>7812499.9999999981</v>
       </c>
-      <c r="G42" s="3">
+      <c r="G44" s="3">
         <v>237</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="H44" s="10" t="s">
         <v>579</v>
       </c>
-      <c r="I42" s="12">
+      <c r="I44" s="12">
         <v>12499999.999999998</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43" s="16" t="s">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45" s="16" t="s">
         <v>521</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="B45" s="17" t="s">
         <v>540</v>
       </c>
-      <c r="C43" s="26">
+      <c r="C45" s="23">
         <v>176000000</v>
       </c>
-      <c r="D43" s="5">
-        <f>I43/1.12</f>
+      <c r="D45" s="5">
+        <f t="shared" si="7"/>
         <v>12053571.428571427</v>
       </c>
-      <c r="E43" s="5">
-        <f>D43*90%</f>
+      <c r="E45" s="5">
+        <f t="shared" si="8"/>
         <v>10848214.285714285</v>
       </c>
-      <c r="F43" s="5">
-        <f>D43*70%</f>
+      <c r="F45" s="5">
+        <f t="shared" si="9"/>
         <v>8437499.9999999981</v>
       </c>
-      <c r="G43" s="27">
+      <c r="G45" s="24">
         <v>238</v>
       </c>
-      <c r="H43" s="16" t="s">
+      <c r="H45" s="16" t="s">
         <v>579</v>
       </c>
-      <c r="I43" s="19">
+      <c r="I45" s="19">
         <v>13500000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A44" s="4" t="s">
-        <v>529</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>539</v>
-      </c>
-      <c r="C44" s="5">
-        <v>155700000</v>
-      </c>
-      <c r="D44" s="5">
-        <f>I44/1.12</f>
-        <v>10892857.142857142</v>
-      </c>
-      <c r="E44" s="5">
-        <f>D44*90%</f>
-        <v>9803571.4285714272</v>
-      </c>
-      <c r="F44" s="5">
-        <f>D44*70%</f>
-        <v>7624999.9999999991</v>
-      </c>
-      <c r="G44" s="3">
-        <v>201</v>
-      </c>
-      <c r="H44" s="4" t="s">
-        <v>572</v>
-      </c>
-      <c r="I44" s="12">
-        <v>12200000</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A45" s="4" t="s">
-        <v>609</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>610</v>
-      </c>
-      <c r="C45" s="9">
-        <v>167800000</v>
-      </c>
-      <c r="D45" s="9">
-        <f>I45/1.12</f>
-        <v>7142857.1428571418</v>
-      </c>
-      <c r="E45" s="9">
-        <f>D45*90%</f>
-        <v>6428571.4285714282</v>
-      </c>
-      <c r="F45" s="9">
-        <f>D45*70%</f>
-        <v>4999999.9999999991</v>
-      </c>
-      <c r="G45" s="20">
-        <v>229</v>
-      </c>
-      <c r="H45" s="4" t="s">
-        <v>572</v>
-      </c>
-      <c r="I45" s="12">
-        <v>8000000</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
-        <v>520</v>
+        <v>529</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>513</v>
+        <v>539</v>
       </c>
       <c r="C46" s="5">
-        <v>172600000</v>
+        <v>155700000</v>
       </c>
       <c r="D46" s="5">
-        <f>I46/1.12</f>
-        <v>7142857.1428571418</v>
+        <f t="shared" si="7"/>
+        <v>10892857.142857142</v>
       </c>
       <c r="E46" s="5">
-        <f>D46*90%</f>
-        <v>6428571.4285714282</v>
+        <f t="shared" si="8"/>
+        <v>9803571.4285714272</v>
       </c>
       <c r="F46" s="5">
-        <f>D46*70%</f>
-        <v>4999999.9999999991</v>
+        <f t="shared" si="9"/>
+        <v>7624999.9999999991</v>
       </c>
       <c r="G46" s="3">
-        <v>230</v>
+        <v>201</v>
       </c>
       <c r="H46" s="4" t="s">
         <v>572</v>
       </c>
       <c r="I46" s="12">
+        <v>12200000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A47" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="C47" s="9">
+        <v>167800000</v>
+      </c>
+      <c r="D47" s="9">
+        <f t="shared" si="7"/>
+        <v>7142857.1428571418</v>
+      </c>
+      <c r="E47" s="9">
+        <f t="shared" si="8"/>
+        <v>6428571.4285714282</v>
+      </c>
+      <c r="F47" s="9">
+        <f t="shared" si="9"/>
+        <v>4999999.9999999991</v>
+      </c>
+      <c r="G47" s="20">
+        <v>229</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="I47" s="12">
         <v>8000000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A47" s="17" t="s">
-        <v>593</v>
-      </c>
-      <c r="B47" s="17" t="s">
-        <v>589</v>
-      </c>
-      <c r="C47" s="18">
-        <v>328000000</v>
-      </c>
-      <c r="D47" s="18">
-        <f>I47/1.12</f>
-        <v>17857142.857142854</v>
-      </c>
-      <c r="E47" s="18">
-        <f>D47*90%</f>
-        <v>16071428.571428569</v>
-      </c>
-      <c r="F47" s="18">
-        <f>D47*70%</f>
-        <v>12499999.999999998</v>
-      </c>
-      <c r="G47" s="21">
-        <v>254</v>
-      </c>
-      <c r="H47" s="17" t="s">
-        <v>593</v>
-      </c>
-      <c r="I47" s="19">
-        <v>20000000</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
-        <v>604</v>
+        <v>520</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>589</v>
-      </c>
-      <c r="C48" s="9">
-        <v>328000000</v>
-      </c>
-      <c r="D48" s="9">
-        <f>I48/1.12</f>
-        <v>17857142.857142854</v>
-      </c>
-      <c r="E48" s="9">
-        <f>D48*90%</f>
-        <v>16071428.571428569</v>
-      </c>
-      <c r="F48" s="9">
-        <f>D48*70%</f>
-        <v>12499999.999999998</v>
-      </c>
-      <c r="G48" s="20">
-        <v>254</v>
+        <v>513</v>
+      </c>
+      <c r="C48" s="5">
+        <v>172600000</v>
+      </c>
+      <c r="D48" s="5">
+        <f t="shared" si="7"/>
+        <v>7142857.1428571418</v>
+      </c>
+      <c r="E48" s="5">
+        <f t="shared" si="8"/>
+        <v>6428571.4285714282</v>
+      </c>
+      <c r="F48" s="5">
+        <f t="shared" si="9"/>
+        <v>4999999.9999999991</v>
+      </c>
+      <c r="G48" s="3">
+        <v>230</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>593</v>
+        <v>572</v>
       </c>
       <c r="I48" s="12">
-        <v>20000000</v>
+        <v>8000000</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" s="17" t="s">
-        <v>595</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>591</v>
-      </c>
-      <c r="C49" s="9">
-        <v>358000000</v>
-      </c>
-      <c r="D49" s="9">
-        <f>I49/1.12</f>
-        <v>22321428.571428571</v>
-      </c>
-      <c r="E49" s="9">
-        <f>D49*90%</f>
-        <v>20089285.714285713</v>
-      </c>
-      <c r="F49" s="9">
-        <f>D49*70%</f>
-        <v>15624999.999999998</v>
-      </c>
-      <c r="G49" s="20">
-        <v>255</v>
-      </c>
-      <c r="H49" s="4" t="s">
-        <v>595</v>
-      </c>
-      <c r="I49" s="12">
-        <v>25000000</v>
+        <v>593</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>589</v>
+      </c>
+      <c r="C49" s="18">
+        <v>328000000</v>
+      </c>
+      <c r="D49" s="18">
+        <f t="shared" si="7"/>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E49" s="18">
+        <f t="shared" si="8"/>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F49" s="18">
+        <f t="shared" si="9"/>
+        <v>12499999.999999998</v>
+      </c>
+      <c r="G49" s="21">
+        <v>254</v>
+      </c>
+      <c r="H49" s="17" t="s">
+        <v>593</v>
+      </c>
+      <c r="I49" s="19">
+        <v>20000000</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C50" s="9">
-        <v>358000000</v>
+        <v>328000000</v>
       </c>
       <c r="D50" s="9">
-        <f>I50/1.12</f>
-        <v>22321428.571428571</v>
+        <f t="shared" si="7"/>
+        <v>17857142.857142854</v>
       </c>
       <c r="E50" s="9">
-        <f>D50*90%</f>
-        <v>20089285.714285713</v>
+        <f t="shared" si="8"/>
+        <v>16071428.571428569</v>
       </c>
       <c r="F50" s="9">
-        <f>D50*70%</f>
-        <v>15624999.999999998</v>
+        <f t="shared" si="9"/>
+        <v>12499999.999999998</v>
       </c>
       <c r="G50" s="20">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="I50" s="12">
-        <v>25000000</v>
+        <v>20000000</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" s="17" t="s">
+        <v>595</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="C51" s="9">
+        <v>358000000</v>
+      </c>
+      <c r="D51" s="9">
+        <f t="shared" si="7"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E51" s="9">
+        <f t="shared" si="8"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F51" s="9">
+        <f t="shared" si="9"/>
+        <v>15624999.999999998</v>
+      </c>
+      <c r="G51" s="20">
+        <v>255</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>595</v>
+      </c>
+      <c r="I51" s="12">
+        <v>25000000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A52" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="C52" s="9">
+        <v>358000000</v>
+      </c>
+      <c r="D52" s="9">
+        <f t="shared" si="7"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E52" s="9">
+        <f t="shared" si="8"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F52" s="9">
+        <f t="shared" si="9"/>
+        <v>15624999.999999998</v>
+      </c>
+      <c r="G52" s="20">
+        <v>255</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>595</v>
+      </c>
+      <c r="I52" s="12">
+        <v>25000000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A53" s="17" t="s">
         <v>594</v>
       </c>
-      <c r="B51" s="17" t="s">
+      <c r="B53" s="17" t="s">
         <v>590</v>
       </c>
-      <c r="C51" s="18">
+      <c r="C53" s="18">
         <v>348000000</v>
       </c>
-      <c r="D51" s="18">
-        <f>I51/1.12</f>
+      <c r="D53" s="18">
+        <f t="shared" si="7"/>
         <v>17857142.857142854</v>
       </c>
-      <c r="E51" s="18">
-        <f>D51*90%</f>
+      <c r="E53" s="18">
+        <f t="shared" si="8"/>
         <v>16071428.571428569</v>
       </c>
-      <c r="F51" s="18">
-        <f>D51*70%</f>
+      <c r="F53" s="18">
+        <f t="shared" si="9"/>
         <v>12499999.999999998</v>
       </c>
-      <c r="G51" s="21">
+      <c r="G53" s="21">
         <v>256</v>
       </c>
-      <c r="H51" s="17" t="s">
+      <c r="H53" s="17" t="s">
         <v>594</v>
       </c>
-      <c r="I51" s="19">
+      <c r="I53" s="19">
         <v>20000000</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A52" s="16" t="s">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A54" s="16" t="s">
         <v>606</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B54" s="4" t="s">
         <v>590</v>
       </c>
-      <c r="C52" s="18">
+      <c r="C54" s="18">
         <v>348000000</v>
       </c>
-      <c r="D52" s="18">
-        <f>I52/1.12</f>
+      <c r="D54" s="18">
+        <f t="shared" si="7"/>
         <v>17857142.857142854</v>
       </c>
-      <c r="E52" s="18">
-        <f>D52*90%</f>
+      <c r="E54" s="18">
+        <f t="shared" si="8"/>
         <v>16071428.571428569</v>
       </c>
-      <c r="F52" s="18">
-        <f>D52*70%</f>
+      <c r="F54" s="18">
+        <f t="shared" si="9"/>
         <v>12499999.999999998</v>
       </c>
-      <c r="G52" s="21">
+      <c r="G54" s="21">
         <v>256</v>
       </c>
-      <c r="H52" s="4" t="s">
+      <c r="H54" s="4" t="s">
         <v>594</v>
       </c>
-      <c r="I52" s="12">
+      <c r="I54" s="12">
         <v>20000000</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A53" s="16" t="s">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A55" s="16" t="s">
         <v>596</v>
       </c>
-      <c r="B53" s="17" t="s">
+      <c r="B55" s="17" t="s">
         <v>592</v>
       </c>
-      <c r="C53" s="9">
+      <c r="C55" s="9">
         <v>378000000</v>
       </c>
-      <c r="D53" s="9">
-        <f>I53/1.12</f>
+      <c r="D55" s="9">
+        <f t="shared" si="7"/>
         <v>22321428.571428571</v>
       </c>
-      <c r="E53" s="9">
-        <f>D53*90%</f>
+      <c r="E55" s="9">
+        <f t="shared" si="8"/>
         <v>20089285.714285713</v>
       </c>
-      <c r="F53" s="9">
-        <f>D53*70%</f>
+      <c r="F55" s="9">
+        <f t="shared" si="9"/>
         <v>15624999.999999998</v>
       </c>
-      <c r="G53" s="20">
+      <c r="G55" s="20">
         <v>257</v>
       </c>
-      <c r="H53" s="4" t="s">
+      <c r="H55" s="4" t="s">
         <v>596</v>
       </c>
-      <c r="I53" s="12">
+      <c r="I55" s="12">
         <v>25000000</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A54" s="4" t="s">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56" s="4" t="s">
         <v>605</v>
       </c>
-      <c r="B54" s="17" t="s">
+      <c r="B56" s="17" t="s">
         <v>592</v>
       </c>
-      <c r="C54" s="18">
+      <c r="C56" s="18">
         <v>378000000</v>
       </c>
-      <c r="D54" s="9">
-        <f>I54/1.12</f>
+      <c r="D56" s="9">
+        <f t="shared" si="7"/>
         <v>22321428.571428571</v>
       </c>
-      <c r="E54" s="9">
-        <f>D54*90%</f>
+      <c r="E56" s="9">
+        <f t="shared" si="8"/>
         <v>20089285.714285713</v>
       </c>
-      <c r="F54" s="9">
-        <f>D54*70%</f>
+      <c r="F56" s="9">
+        <f t="shared" si="9"/>
         <v>15624999.999999998</v>
       </c>
-      <c r="G54" s="21">
+      <c r="G56" s="21">
         <v>257</v>
       </c>
-      <c r="H54" s="17" t="s">
+      <c r="H56" s="17" t="s">
         <v>596</v>
       </c>
-      <c r="I54" s="19">
+      <c r="I56" s="19">
         <v>25000000</v>
       </c>
     </row>
@@ -7415,17 +7490,17 @@
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A29 A31:A43">
+  <conditionalFormatting sqref="A33:A45 A2:A31">
     <cfRule type="duplicateValues" dxfId="7" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A31:A38 A2:A29 A40:A43">
+  <conditionalFormatting sqref="A33:A40 A42:A45 A2:A31">
     <cfRule type="duplicateValues" dxfId="6" priority="13"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H40:H43">
+  <conditionalFormatting sqref="H42:H45">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
     <cfRule type="duplicateValues" dxfId="4" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H48:H51">
+  <conditionalFormatting sqref="H50:H53">
     <cfRule type="duplicateValues" dxfId="3" priority="2"/>
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Added NEW CORTEZ CE to pricelist
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3CFD31-6A96-46C9-A31C-BE51EF926D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06DF8933-CC8E-49B7-8963-B419AF88E07C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -490,7 +490,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="619">
   <si>
     <t>Column1</t>
   </si>
@@ -2424,6 +2424,9 @@
   </si>
   <si>
     <t>New Alvez EX AT</t>
+  </si>
+  <si>
+    <t>NEW CORTEZ CE LUX +CVT</t>
   </si>
 </sst>
 </file>
@@ -2615,7 +2618,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2658,7 +2661,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -5033,10 +5035,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I56" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
-  <autoFilter ref="A1:I56" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I56">
-    <sortCondition ref="H1:H56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I57" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
+  <autoFilter ref="A1:I57" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I57">
+    <sortCondition ref="H1:H57"/>
   </sortState>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="149"/>
@@ -5662,7 +5664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B05C9E0-A64E-40AC-B9F4-C919ED5906CC}">
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
@@ -6207,7 +6209,7 @@
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="10" t="s">
         <v>613</v>
       </c>
       <c r="B17" s="4" t="s">
@@ -6239,7 +6241,7 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="10" t="s">
         <v>616</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -6266,7 +6268,7 @@
       <c r="H18" s="4" t="s">
         <v>566</v>
       </c>
-      <c r="I18" s="26">
+      <c r="I18" s="12">
         <v>23000000</v>
       </c>
     </row>
@@ -6825,15 +6827,15 @@
         <v>291300000</v>
       </c>
       <c r="D36" s="5">
-        <f t="shared" ref="D36:D56" si="7">I36/1.12</f>
+        <f t="shared" ref="D36:D57" si="7">I36/1.12</f>
         <v>19642857.142857142</v>
       </c>
       <c r="E36" s="5">
-        <f t="shared" ref="E36:E67" si="8">D36*90%</f>
+        <f t="shared" ref="E36:E57" si="8">D36*90%</f>
         <v>17678571.428571429</v>
       </c>
       <c r="F36" s="5">
-        <f t="shared" ref="F36:F56" si="9">D36*70%</f>
+        <f t="shared" ref="F36:F57" si="9">D36*70%</f>
         <v>13749999.999999998</v>
       </c>
       <c r="G36" s="3">
@@ -6879,456 +6881,456 @@
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A38" s="11" t="s">
+      <c r="A38" s="25" t="s">
+        <v>618</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>612</v>
+      </c>
+      <c r="C38" s="9">
+        <v>307300000</v>
+      </c>
+      <c r="D38" s="5">
+        <f t="shared" ref="D38" si="10">I38/1.12</f>
+        <v>19999999.999999996</v>
+      </c>
+      <c r="E38" s="5">
+        <f t="shared" ref="E38" si="11">D38*90%</f>
+        <v>17999999.999999996</v>
+      </c>
+      <c r="F38" s="5">
+        <f t="shared" ref="F38" si="12">D38*70%</f>
+        <v>13999999.999999996</v>
+      </c>
+      <c r="G38" s="20">
+        <v>210</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="I38" s="12">
+        <v>22400000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="11" t="s">
         <v>522</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B39" s="4" t="s">
         <v>550</v>
       </c>
-      <c r="C38" s="5">
+      <c r="C39" s="5">
         <v>345650000</v>
       </c>
-      <c r="D38" s="5">
+      <c r="D39" s="5">
         <f t="shared" si="7"/>
         <v>22857142.857142854</v>
       </c>
-      <c r="E38" s="5">
+      <c r="E39" s="5">
         <f t="shared" si="8"/>
         <v>20571428.571428571</v>
       </c>
-      <c r="F38" s="5">
+      <c r="F39" s="5">
         <f t="shared" si="9"/>
         <v>15999999.999999996</v>
       </c>
-      <c r="G38" s="3">
+      <c r="G39" s="3">
         <v>233</v>
       </c>
-      <c r="H38" s="4" t="s">
+      <c r="H39" s="4" t="s">
         <v>567</v>
       </c>
-      <c r="I38" s="12">
+      <c r="I39" s="12">
         <v>25600000</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A39" s="22" t="s">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B40" s="4" t="s">
         <v>612</v>
       </c>
-      <c r="C39" s="9">
+      <c r="C40" s="9">
         <v>307300000</v>
       </c>
-      <c r="D39" s="5">
+      <c r="D40" s="5">
         <f t="shared" si="7"/>
         <v>19999999.999999996</v>
       </c>
-      <c r="E39" s="5">
+      <c r="E40" s="5">
         <f t="shared" si="8"/>
         <v>17999999.999999996</v>
       </c>
-      <c r="F39" s="5">
+      <c r="F40" s="5">
         <f t="shared" si="9"/>
         <v>13999999.999999996</v>
       </c>
-      <c r="G39" s="4">
+      <c r="G40" s="20">
         <v>210</v>
       </c>
-      <c r="H39" s="4" t="s">
+      <c r="H40" s="4" t="s">
         <v>567</v>
       </c>
-      <c r="I39" s="12">
+      <c r="I40" s="12">
         <v>22400000</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A40" s="10" t="s">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" s="10" t="s">
         <v>608</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B41" s="4" t="s">
         <v>597</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C41" s="9">
         <v>399000000</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D41" s="9">
         <f t="shared" si="7"/>
         <v>28214285.714285713</v>
       </c>
-      <c r="E40" s="9">
+      <c r="E41" s="9">
         <f t="shared" si="8"/>
         <v>25392857.142857142</v>
       </c>
-      <c r="F40" s="9">
+      <c r="F41" s="9">
         <f t="shared" si="9"/>
         <v>19749999.999999996</v>
       </c>
-      <c r="G40" s="20">
+      <c r="G41" s="20">
         <v>258</v>
       </c>
-      <c r="H40" s="4" t="s">
+      <c r="H41" s="4" t="s">
         <v>597</v>
       </c>
-      <c r="I40" s="12">
+      <c r="I41" s="12">
         <v>31600000</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A41" s="10" t="s">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42" s="10" t="s">
         <v>599</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B42" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C42" s="9">
         <v>459000000</v>
       </c>
-      <c r="D41" s="9">
+      <c r="D42" s="9">
         <f t="shared" si="7"/>
         <v>32499999.999999996</v>
       </c>
-      <c r="E41" s="9">
+      <c r="E42" s="9">
         <f t="shared" si="8"/>
         <v>29249999.999999996</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F42" s="9">
         <f t="shared" si="9"/>
         <v>22749999.999999996</v>
       </c>
-      <c r="G41" s="20">
+      <c r="G42" s="20">
         <v>259</v>
       </c>
-      <c r="H41" s="4" t="s">
+      <c r="H42" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="I41" s="12">
+      <c r="I42" s="12">
         <v>36400000</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A42" s="10" t="s">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43" s="10" t="s">
         <v>601</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B43" s="4" t="s">
         <v>600</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C43" s="9">
         <v>449000000</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D43" s="9">
         <f t="shared" si="7"/>
         <v>29196428.571428567</v>
       </c>
-      <c r="E42" s="9">
+      <c r="E43" s="9">
         <f t="shared" si="8"/>
         <v>26276785.714285713</v>
       </c>
-      <c r="F42" s="9">
+      <c r="F43" s="9">
         <f t="shared" si="9"/>
         <v>20437499.999999996</v>
       </c>
-      <c r="G42" s="20">
+      <c r="G43" s="20">
         <v>260</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="H43" s="10" t="s">
         <v>600</v>
       </c>
-      <c r="I42" s="12">
+      <c r="I43" s="12">
         <v>32700000</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43" s="10" t="s">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44" s="10" t="s">
         <v>603</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B44" s="4" t="s">
         <v>602</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C44" s="9">
         <v>499000000</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D44" s="9">
         <f t="shared" si="7"/>
         <v>32499999.999999996</v>
       </c>
-      <c r="E43" s="9">
+      <c r="E44" s="9">
         <f t="shared" si="8"/>
         <v>29249999.999999996</v>
       </c>
-      <c r="F43" s="9">
+      <c r="F44" s="9">
         <f t="shared" si="9"/>
         <v>22749999.999999996</v>
       </c>
-      <c r="G43" s="20">
+      <c r="G44" s="20">
         <v>261</v>
       </c>
-      <c r="H43" s="10" t="s">
+      <c r="H44" s="10" t="s">
         <v>602</v>
       </c>
-      <c r="I43" s="12">
+      <c r="I44" s="12">
         <v>36400000</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A44" s="10" t="s">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45" s="10" t="s">
         <v>526</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B45" s="4" t="s">
         <v>545</v>
       </c>
-      <c r="C44" s="5">
+      <c r="C45" s="5">
         <v>168000000</v>
       </c>
-      <c r="D44" s="5">
+      <c r="D45" s="5">
         <f t="shared" si="7"/>
         <v>11160714.285714284</v>
       </c>
-      <c r="E44" s="5">
+      <c r="E45" s="5">
         <f t="shared" si="8"/>
         <v>10044642.857142856</v>
       </c>
-      <c r="F44" s="5">
+      <c r="F45" s="5">
         <f t="shared" si="9"/>
         <v>7812499.9999999981</v>
       </c>
-      <c r="G44" s="3">
+      <c r="G45" s="3">
         <v>237</v>
       </c>
-      <c r="H44" s="10" t="s">
+      <c r="H45" s="10" t="s">
         <v>579</v>
       </c>
-      <c r="I44" s="12">
+      <c r="I45" s="12">
         <v>12499999.999999998</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A45" s="16" t="s">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A46" s="16" t="s">
         <v>521</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="B46" s="17" t="s">
         <v>540</v>
       </c>
-      <c r="C45" s="23">
+      <c r="C46" s="23">
         <v>176000000</v>
       </c>
-      <c r="D45" s="5">
+      <c r="D46" s="5">
         <f t="shared" si="7"/>
         <v>12053571.428571427</v>
       </c>
-      <c r="E45" s="5">
+      <c r="E46" s="5">
         <f t="shared" si="8"/>
         <v>10848214.285714285</v>
       </c>
-      <c r="F45" s="5">
+      <c r="F46" s="5">
         <f t="shared" si="9"/>
         <v>8437499.9999999981</v>
       </c>
-      <c r="G45" s="24">
+      <c r="G46" s="24">
         <v>238</v>
       </c>
-      <c r="H45" s="16" t="s">
+      <c r="H46" s="16" t="s">
         <v>579</v>
       </c>
-      <c r="I45" s="19">
+      <c r="I46" s="19">
         <v>13500000</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A46" s="4" t="s">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A47" s="4" t="s">
         <v>529</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B47" s="4" t="s">
         <v>539</v>
       </c>
-      <c r="C46" s="5">
+      <c r="C47" s="5">
         <v>155700000</v>
       </c>
-      <c r="D46" s="5">
+      <c r="D47" s="5">
         <f t="shared" si="7"/>
         <v>10892857.142857142</v>
       </c>
-      <c r="E46" s="5">
+      <c r="E47" s="5">
         <f t="shared" si="8"/>
         <v>9803571.4285714272</v>
       </c>
-      <c r="F46" s="5">
+      <c r="F47" s="5">
         <f t="shared" si="9"/>
         <v>7624999.9999999991</v>
       </c>
-      <c r="G46" s="3">
+      <c r="G47" s="3">
         <v>201</v>
       </c>
-      <c r="H46" s="4" t="s">
+      <c r="H47" s="4" t="s">
         <v>572</v>
       </c>
-      <c r="I46" s="12">
+      <c r="I47" s="12">
         <v>12200000</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A47" s="4" t="s">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A48" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B48" s="4" t="s">
         <v>610</v>
       </c>
-      <c r="C47" s="9">
+      <c r="C48" s="9">
         <v>167800000</v>
       </c>
-      <c r="D47" s="9">
+      <c r="D48" s="9">
         <f t="shared" si="7"/>
         <v>7142857.1428571418</v>
       </c>
-      <c r="E47" s="9">
+      <c r="E48" s="9">
         <f t="shared" si="8"/>
         <v>6428571.4285714282</v>
       </c>
-      <c r="F47" s="9">
+      <c r="F48" s="9">
         <f t="shared" si="9"/>
         <v>4999999.9999999991</v>
       </c>
-      <c r="G47" s="20">
+      <c r="G48" s="20">
         <v>229</v>
       </c>
-      <c r="H47" s="4" t="s">
+      <c r="H48" s="4" t="s">
         <v>572</v>
       </c>
-      <c r="I47" s="12">
+      <c r="I48" s="12">
         <v>8000000</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="4" t="s">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A49" s="4" t="s">
         <v>520</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B49" s="4" t="s">
         <v>513</v>
       </c>
-      <c r="C48" s="5">
+      <c r="C49" s="5">
         <v>172600000</v>
       </c>
-      <c r="D48" s="5">
+      <c r="D49" s="5">
         <f t="shared" si="7"/>
         <v>7142857.1428571418</v>
       </c>
-      <c r="E48" s="5">
+      <c r="E49" s="5">
         <f t="shared" si="8"/>
         <v>6428571.4285714282</v>
       </c>
-      <c r="F48" s="5">
+      <c r="F49" s="5">
         <f t="shared" si="9"/>
         <v>4999999.9999999991</v>
       </c>
-      <c r="G48" s="3">
+      <c r="G49" s="3">
         <v>230</v>
       </c>
-      <c r="H48" s="4" t="s">
+      <c r="H49" s="4" t="s">
         <v>572</v>
       </c>
-      <c r="I48" s="12">
+      <c r="I49" s="12">
         <v>8000000</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A49" s="17" t="s">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A50" s="17" t="s">
         <v>593</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B50" s="17" t="s">
         <v>589</v>
       </c>
-      <c r="C49" s="18">
+      <c r="C50" s="18">
         <v>328000000</v>
       </c>
-      <c r="D49" s="18">
+      <c r="D50" s="18">
         <f t="shared" si="7"/>
         <v>17857142.857142854</v>
       </c>
-      <c r="E49" s="18">
+      <c r="E50" s="18">
         <f t="shared" si="8"/>
         <v>16071428.571428569</v>
       </c>
-      <c r="F49" s="18">
+      <c r="F50" s="18">
         <f t="shared" si="9"/>
         <v>12499999.999999998</v>
       </c>
-      <c r="G49" s="21">
+      <c r="G50" s="21">
         <v>254</v>
       </c>
-      <c r="H49" s="17" t="s">
+      <c r="H50" s="17" t="s">
         <v>593</v>
       </c>
-      <c r="I49" s="19">
+      <c r="I50" s="19">
         <v>20000000</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A50" s="4" t="s">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A51" s="4" t="s">
         <v>604</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B51" s="4" t="s">
         <v>589</v>
       </c>
-      <c r="C50" s="9">
+      <c r="C51" s="9">
         <v>328000000</v>
       </c>
-      <c r="D50" s="9">
+      <c r="D51" s="9">
         <f t="shared" si="7"/>
         <v>17857142.857142854</v>
       </c>
-      <c r="E50" s="9">
+      <c r="E51" s="9">
         <f t="shared" si="8"/>
         <v>16071428.571428569</v>
       </c>
-      <c r="F50" s="9">
+      <c r="F51" s="9">
         <f t="shared" si="9"/>
         <v>12499999.999999998</v>
       </c>
-      <c r="G50" s="20">
+      <c r="G51" s="20">
         <v>254</v>
       </c>
-      <c r="H50" s="4" t="s">
+      <c r="H51" s="4" t="s">
         <v>593</v>
       </c>
-      <c r="I50" s="12">
+      <c r="I51" s="12">
         <v>20000000</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A51" s="17" t="s">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A52" s="17" t="s">
         <v>595</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>591</v>
-      </c>
-      <c r="C51" s="9">
-        <v>358000000</v>
-      </c>
-      <c r="D51" s="9">
-        <f t="shared" si="7"/>
-        <v>22321428.571428571</v>
-      </c>
-      <c r="E51" s="9">
-        <f t="shared" si="8"/>
-        <v>20089285.714285713</v>
-      </c>
-      <c r="F51" s="9">
-        <f t="shared" si="9"/>
-        <v>15624999.999999998</v>
-      </c>
-      <c r="G51" s="20">
-        <v>255</v>
-      </c>
-      <c r="H51" s="4" t="s">
-        <v>595</v>
-      </c>
-      <c r="I51" s="12">
-        <v>25000000</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A52" s="4" t="s">
-        <v>607</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>591</v>
@@ -7359,42 +7361,42 @@
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A53" s="17" t="s">
+      <c r="A53" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="C53" s="9">
+        <v>358000000</v>
+      </c>
+      <c r="D53" s="9">
+        <f t="shared" si="7"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E53" s="9">
+        <f t="shared" si="8"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F53" s="9">
+        <f t="shared" si="9"/>
+        <v>15624999.999999998</v>
+      </c>
+      <c r="G53" s="20">
+        <v>255</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>595</v>
+      </c>
+      <c r="I53" s="12">
+        <v>25000000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A54" s="17" t="s">
         <v>594</v>
       </c>
-      <c r="B53" s="17" t="s">
-        <v>590</v>
-      </c>
-      <c r="C53" s="18">
-        <v>348000000</v>
-      </c>
-      <c r="D53" s="18">
-        <f t="shared" si="7"/>
-        <v>17857142.857142854</v>
-      </c>
-      <c r="E53" s="18">
-        <f t="shared" si="8"/>
-        <v>16071428.571428569</v>
-      </c>
-      <c r="F53" s="18">
-        <f t="shared" si="9"/>
-        <v>12499999.999999998</v>
-      </c>
-      <c r="G53" s="21">
-        <v>256</v>
-      </c>
-      <c r="H53" s="17" t="s">
-        <v>594</v>
-      </c>
-      <c r="I53" s="19">
-        <v>20000000</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A54" s="16" t="s">
-        <v>606</v>
-      </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="17" t="s">
         <v>590</v>
       </c>
       <c r="C54" s="18">
@@ -7415,53 +7417,53 @@
       <c r="G54" s="21">
         <v>256</v>
       </c>
-      <c r="H54" s="4" t="s">
+      <c r="H54" s="17" t="s">
         <v>594</v>
       </c>
-      <c r="I54" s="12">
+      <c r="I54" s="19">
         <v>20000000</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" s="16" t="s">
+        <v>606</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C55" s="18">
+        <v>348000000</v>
+      </c>
+      <c r="D55" s="18">
+        <f t="shared" si="7"/>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E55" s="18">
+        <f t="shared" si="8"/>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F55" s="18">
+        <f t="shared" si="9"/>
+        <v>12499999.999999998</v>
+      </c>
+      <c r="G55" s="21">
+        <v>256</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="I55" s="12">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56" s="16" t="s">
         <v>596</v>
-      </c>
-      <c r="B55" s="17" t="s">
-        <v>592</v>
-      </c>
-      <c r="C55" s="9">
-        <v>378000000</v>
-      </c>
-      <c r="D55" s="9">
-        <f t="shared" si="7"/>
-        <v>22321428.571428571</v>
-      </c>
-      <c r="E55" s="9">
-        <f t="shared" si="8"/>
-        <v>20089285.714285713</v>
-      </c>
-      <c r="F55" s="9">
-        <f t="shared" si="9"/>
-        <v>15624999.999999998</v>
-      </c>
-      <c r="G55" s="20">
-        <v>257</v>
-      </c>
-      <c r="H55" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="I55" s="12">
-        <v>25000000</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A56" s="4" t="s">
-        <v>605</v>
       </c>
       <c r="B56" s="17" t="s">
         <v>592</v>
       </c>
-      <c r="C56" s="18">
+      <c r="C56" s="9">
         <v>378000000</v>
       </c>
       <c r="D56" s="9">
@@ -7476,13 +7478,45 @@
         <f t="shared" si="9"/>
         <v>15624999.999999998</v>
       </c>
-      <c r="G56" s="21">
+      <c r="G56" s="20">
         <v>257</v>
       </c>
-      <c r="H56" s="17" t="s">
+      <c r="H56" s="4" t="s">
         <v>596</v>
       </c>
-      <c r="I56" s="19">
+      <c r="I56" s="12">
+        <v>25000000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A57" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="B57" s="17" t="s">
+        <v>592</v>
+      </c>
+      <c r="C57" s="18">
+        <v>378000000</v>
+      </c>
+      <c r="D57" s="9">
+        <f t="shared" si="7"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E57" s="9">
+        <f t="shared" si="8"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F57" s="9">
+        <f t="shared" si="9"/>
+        <v>15624999.999999998</v>
+      </c>
+      <c r="G57" s="21">
+        <v>257</v>
+      </c>
+      <c r="H57" s="17" t="s">
+        <v>596</v>
+      </c>
+      <c r="I57" s="19">
         <v>25000000</v>
       </c>
     </row>
@@ -7490,17 +7524,17 @@
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A33:A45 A2:A31">
-    <cfRule type="duplicateValues" dxfId="7" priority="17"/>
+  <conditionalFormatting sqref="A33:A41 A43:A46 A2:A31">
+    <cfRule type="duplicateValues" dxfId="7" priority="13"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A33:A40 A42:A45 A2:A31">
-    <cfRule type="duplicateValues" dxfId="6" priority="13"/>
+  <conditionalFormatting sqref="A33:A46 A2:A31">
+    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H42:H45">
+  <conditionalFormatting sqref="H43:H46">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
     <cfRule type="duplicateValues" dxfId="4" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H50:H53">
+  <conditionalFormatting sqref="H51:H54">
     <cfRule type="duplicateValues" dxfId="3" priority="2"/>
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
UPDATE: Corrected New Alvez EX name in pricelist
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED8C7D2-EDB9-452F-8CF8-F6A6489EE104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC6028A-8AAC-48A7-B53E-7A08AAE2BC43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -2420,13 +2420,13 @@
     <t>New Alvez CE AT</t>
   </si>
   <si>
-    <t>NEW ALVEZ CE AT 310S I2D1 (4X2) A/T</t>
-  </si>
-  <si>
     <t>New Alvez EX AT</t>
   </si>
   <si>
     <t>NEW CORTEZ CE LUX +CVT</t>
+  </si>
+  <si>
+    <t>NEW ALVEZ EX AT 310S I2D1 (4X2) A/T</t>
   </si>
 </sst>
 </file>
@@ -2618,7 +2618,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2660,6 +2660,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -5034,8 +5037,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I57" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
-  <autoFilter ref="A1:I57" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I58" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
+  <autoFilter ref="A1:I58" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I57">
     <sortCondition ref="H1:H57"/>
   </sortState>
@@ -5663,7 +5666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B05C9E0-A64E-40AC-B9F4-C919ED5906CC}">
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
@@ -6241,10 +6244,10 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
+        <v>618</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>616</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>617</v>
       </c>
       <c r="C18" s="9">
         <v>303000000</v>
@@ -6881,7 +6884,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>612</v>
@@ -7518,6 +7521,17 @@
       <c r="I57" s="19">
         <v>25000000</v>
       </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A58" s="25"/>
+      <c r="B58" s="26"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="18"/>
+      <c r="G58" s="17"/>
+      <c r="H58" s="17"/>
+      <c r="I58" s="27"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">

</xml_diff>

<commit_message>
UPDATE: Fix pricelist for Darion PHEV LV1 (P3C)
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC6028A-8AAC-48A7-B53E-7A08AAE2BC43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87A99CB-0DE2-4623-9DD9-40C9371FE9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -2375,9 +2375,6 @@
     <t>DARION PHEV LV1</t>
   </si>
   <si>
-    <t>520M P2D (4X2) A/T</t>
-  </si>
-  <si>
     <t>DARION PHEV LV2</t>
   </si>
   <si>
@@ -2427,6 +2424,9 @@
   </si>
   <si>
     <t>NEW ALVEZ EX AT 310S I2D1 (4X2) A/T</t>
+  </si>
+  <si>
+    <t>520M P3C (4X2) A/T</t>
   </si>
 </sst>
 </file>
@@ -2618,7 +2618,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2660,9 +2660,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -6180,10 +6177,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="C16" s="5">
         <v>217000000</v>
@@ -6212,10 +6209,10 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="C17" s="5">
         <v>263000000</v>
@@ -6244,10 +6241,10 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="C18" s="9">
         <v>303000000</v>
@@ -6884,10 +6881,10 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="C38" s="9">
         <v>307300000</v>
@@ -6951,7 +6948,7 @@
         <v>149</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="C40" s="9">
         <v>307300000</v>
@@ -6980,7 +6977,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>597</v>
@@ -7044,7 +7041,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
-        <v>601</v>
+        <v>618</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>600</v>
@@ -7076,10 +7073,10 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="C44" s="9">
         <v>499000000</v>
@@ -7100,7 +7097,7 @@
         <v>261</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="I44" s="12">
         <v>36400000</v>
@@ -7204,10 +7201,10 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="B48" s="4" t="s">
         <v>609</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>610</v>
       </c>
       <c r="C48" s="9">
         <v>167800000</v>
@@ -7300,7 +7297,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>589</v>
@@ -7364,7 +7361,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" s="4" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>591</v>
@@ -7428,7 +7425,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" s="16" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>590</v>
@@ -7492,7 +7489,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" s="4" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B57" s="17" t="s">
         <v>592</v>
@@ -7523,15 +7520,15 @@
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A58" s="25"/>
-      <c r="B58" s="26"/>
+      <c r="A58" s="16"/>
+      <c r="B58" s="17"/>
       <c r="C58" s="18"/>
       <c r="D58" s="18"/>
       <c r="E58" s="18"/>
       <c r="F58" s="18"/>
       <c r="G58" s="17"/>
       <c r="H58" s="17"/>
-      <c r="I58" s="27"/>
+      <c r="I58" s="19"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">

</xml_diff>

<commit_message>
UPDATE: Added EKSION Pricelist
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87A99CB-0DE2-4623-9DD9-40C9371FE9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EFE44EB-1462-4830-B9BF-68AC98C79D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -490,7 +490,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1408" uniqueCount="631">
   <si>
     <t>Column1</t>
   </si>
@@ -2427,6 +2427,42 @@
   </si>
   <si>
     <t>520M P3C (4X2) A/T</t>
+  </si>
+  <si>
+    <t>EKSION EV CE</t>
+  </si>
+  <si>
+    <t>EKSION EV EX</t>
+  </si>
+  <si>
+    <t>EKSION PHEV CE</t>
+  </si>
+  <si>
+    <t>EKSION PHEV EX</t>
+  </si>
+  <si>
+    <t>EKSION EV LV1</t>
+  </si>
+  <si>
+    <t>EKSION PHEV LV1</t>
+  </si>
+  <si>
+    <t>EKSION EV LV2</t>
+  </si>
+  <si>
+    <t>EKSION PHEV LV2</t>
+  </si>
+  <si>
+    <t>520S E1D (4X2) A/T</t>
+  </si>
+  <si>
+    <t>520S E1C (4X2) A/T</t>
+  </si>
+  <si>
+    <t>520S P2D (4X2) A/T</t>
+  </si>
+  <si>
+    <t>520S P3D (4X2) A/T</t>
   </si>
 </sst>
 </file>
@@ -5034,8 +5070,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I58" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
-  <autoFilter ref="A1:I58" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I65" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
+  <autoFilter ref="A1:I65" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I57">
     <sortCondition ref="H1:H57"/>
   </sortState>
@@ -5663,7 +5699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B05C9E0-A64E-40AC-B9F4-C919ED5906CC}">
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
@@ -7520,15 +7556,262 @@
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A58" s="16"/>
-      <c r="B58" s="17"/>
-      <c r="C58" s="18"/>
-      <c r="D58" s="18"/>
-      <c r="E58" s="18"/>
-      <c r="F58" s="18"/>
-      <c r="G58" s="17"/>
-      <c r="H58" s="17"/>
-      <c r="I58" s="19"/>
+      <c r="A58" s="16" t="s">
+        <v>619</v>
+      </c>
+      <c r="B58" s="17" t="s">
+        <v>623</v>
+      </c>
+      <c r="C58" s="18">
+        <v>399000000</v>
+      </c>
+      <c r="D58" s="9">
+        <f t="shared" ref="D58:D65" si="13">I58/1.12</f>
+        <v>20089285.714285716</v>
+      </c>
+      <c r="E58" s="9">
+        <f t="shared" ref="E58:E65" si="14">D58*90%</f>
+        <v>18080357.142857146</v>
+      </c>
+      <c r="F58" s="9">
+        <f t="shared" ref="F58:F65" si="15">D58*70%</f>
+        <v>14062500</v>
+      </c>
+      <c r="G58" s="21">
+        <v>262</v>
+      </c>
+      <c r="H58" s="17" t="s">
+        <v>623</v>
+      </c>
+      <c r="I58" s="19">
+        <f>15625000/7*9*1.12</f>
+        <v>22500000.000000004</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A59" s="16" t="s">
+        <v>620</v>
+      </c>
+      <c r="B59" s="17" t="s">
+        <v>625</v>
+      </c>
+      <c r="C59" s="18">
+        <v>469000000</v>
+      </c>
+      <c r="D59" s="9">
+        <f t="shared" si="13"/>
+        <v>28125000</v>
+      </c>
+      <c r="E59" s="9">
+        <f t="shared" si="14"/>
+        <v>25312500</v>
+      </c>
+      <c r="F59" s="9">
+        <f t="shared" si="15"/>
+        <v>19687500</v>
+      </c>
+      <c r="G59" s="21">
+        <v>263</v>
+      </c>
+      <c r="H59" s="17" t="s">
+        <v>625</v>
+      </c>
+      <c r="I59" s="19">
+        <f>21875000/7*9*1.12</f>
+        <v>31500000.000000004</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A60" s="16" t="s">
+        <v>621</v>
+      </c>
+      <c r="B60" s="17" t="s">
+        <v>624</v>
+      </c>
+      <c r="C60" s="18">
+        <v>459000000</v>
+      </c>
+      <c r="D60" s="9">
+        <f t="shared" si="13"/>
+        <v>28125000</v>
+      </c>
+      <c r="E60" s="9">
+        <f t="shared" si="14"/>
+        <v>25312500</v>
+      </c>
+      <c r="F60" s="9">
+        <f t="shared" si="15"/>
+        <v>19687500</v>
+      </c>
+      <c r="G60" s="21">
+        <v>264</v>
+      </c>
+      <c r="H60" s="17" t="s">
+        <v>624</v>
+      </c>
+      <c r="I60" s="19">
+        <f>21875000/7*9*1.12</f>
+        <v>31500000.000000004</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A61" s="16" t="s">
+        <v>622</v>
+      </c>
+      <c r="B61" s="17" t="s">
+        <v>626</v>
+      </c>
+      <c r="C61" s="18">
+        <v>509000000</v>
+      </c>
+      <c r="D61" s="9">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="E61" s="9">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F61" s="9">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="G61" s="21">
+        <v>265</v>
+      </c>
+      <c r="H61" s="17" t="s">
+        <v>626</v>
+      </c>
+      <c r="I61" s="19"/>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A62" s="16" t="s">
+        <v>628</v>
+      </c>
+      <c r="B62" s="17" t="s">
+        <v>623</v>
+      </c>
+      <c r="C62" s="18">
+        <v>399000000</v>
+      </c>
+      <c r="D62" s="9">
+        <f t="shared" si="13"/>
+        <v>20089285.714285716</v>
+      </c>
+      <c r="E62" s="9">
+        <f t="shared" si="14"/>
+        <v>18080357.142857146</v>
+      </c>
+      <c r="F62" s="9">
+        <f t="shared" si="15"/>
+        <v>14062500</v>
+      </c>
+      <c r="G62" s="21">
+        <v>262</v>
+      </c>
+      <c r="H62" s="17" t="s">
+        <v>623</v>
+      </c>
+      <c r="I62" s="19">
+        <f>15625000/7*9*1.12</f>
+        <v>22500000.000000004</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A63" s="16" t="s">
+        <v>627</v>
+      </c>
+      <c r="B63" s="17" t="s">
+        <v>625</v>
+      </c>
+      <c r="C63" s="18">
+        <v>469000000</v>
+      </c>
+      <c r="D63" s="9">
+        <f t="shared" si="13"/>
+        <v>28125000</v>
+      </c>
+      <c r="E63" s="9">
+        <f t="shared" si="14"/>
+        <v>25312500</v>
+      </c>
+      <c r="F63" s="9">
+        <f t="shared" si="15"/>
+        <v>19687500</v>
+      </c>
+      <c r="G63" s="21">
+        <v>263</v>
+      </c>
+      <c r="H63" s="17" t="s">
+        <v>625</v>
+      </c>
+      <c r="I63" s="19">
+        <f>21875000/7*9*1.12</f>
+        <v>31500000.000000004</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A64" s="16" t="s">
+        <v>629</v>
+      </c>
+      <c r="B64" s="17" t="s">
+        <v>624</v>
+      </c>
+      <c r="C64" s="18">
+        <v>459000000</v>
+      </c>
+      <c r="D64" s="9">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="E64" s="9">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F64" s="9">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="G64" s="21">
+        <v>264</v>
+      </c>
+      <c r="H64" s="17" t="s">
+        <v>624</v>
+      </c>
+      <c r="I64" s="19"/>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A65" s="16" t="s">
+        <v>630</v>
+      </c>
+      <c r="B65" s="17" t="s">
+        <v>626</v>
+      </c>
+      <c r="C65" s="18">
+        <v>509000000</v>
+      </c>
+      <c r="D65" s="9">
+        <f t="shared" si="13"/>
+        <v>28125000</v>
+      </c>
+      <c r="E65" s="9">
+        <f t="shared" si="14"/>
+        <v>25312500</v>
+      </c>
+      <c r="F65" s="9">
+        <f t="shared" si="15"/>
+        <v>19687500</v>
+      </c>
+      <c r="G65" s="21">
+        <v>265</v>
+      </c>
+      <c r="H65" s="17" t="s">
+        <v>626</v>
+      </c>
+      <c r="I65" s="19">
+        <f>21875000/7*9*1.12</f>
+        <v>31500000.000000004</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">

</xml_diff>